<commit_message>
Add README, add events as example.
</commit_message>
<xml_diff>
--- a/events.xlsx
+++ b/events.xlsx
@@ -19,9 +19,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="hh:mm"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -477,7 +478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -541,49 +542,49 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>shift-rome</t>
+          <t>meeting-1</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Morning station shift</t>
+          <t>Planning</t>
         </is>
       </c>
       <c r="C2" s="2" t="b">
         <v>0</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>46237</v>
+        <v>46223</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.3958333333333333</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>46237</v>
+        <v>46223</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>0.5833333333333334</v>
+        <v>0.4375</v>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Roma Termini</t>
+          <t>Office</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Valid timed event</t>
+          <t>Weekly planning</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>holiday-001</t>
+          <t>holiday-1</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Company holiday</t>
+          <t>Holiday</t>
         </is>
       </c>
       <c r="C3" s="2" t="b">
@@ -598,250 +599,7 @@
       </c>
       <c r="G3" s="4" t="n"/>
       <c r="H3" s="2" t="n"/>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>Valid one-day all-day event</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>night-001</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Night maintenance</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="D4" s="3" t="n">
-        <v>46254</v>
-      </c>
-      <c r="E4" s="4" t="n">
-        <v>0.9166666666666666</v>
-      </c>
-      <c r="F4" s="3" t="n">
-        <v>46255</v>
-      </c>
-      <c r="G4" s="4" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>Operations center</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>Valid overnight event</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>conference-001</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Annual conference</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="D5" s="3" t="n">
-        <v>46275</v>
-      </c>
-      <c r="E5" s="4" t="n"/>
-      <c r="F5" s="3" t="n">
-        <v>46277</v>
-      </c>
-      <c r="G5" s="4" t="n"/>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>Convention center</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>Valid multi-day all-day event</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="5" t="n"/>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>Missing identifier</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="D6" s="6" t="n">
-        <v>46239</v>
-      </c>
-      <c r="E6" s="7" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="F6" s="6" t="n">
-        <v>46239</v>
-      </c>
-      <c r="G6" s="7" t="n">
-        <v>0.4166666666666667</v>
-      </c>
-      <c r="H6" s="5" t="inlineStr">
-        <is>
-          <t>Office</t>
-        </is>
-      </c>
-      <c r="I6" s="5" t="inlineStr">
-        <is>
-          <t>Invalid: empty ID</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>missing-summary</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="n"/>
-      <c r="C7" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="D7" s="6" t="n">
-        <v>46240</v>
-      </c>
-      <c r="E7" s="7" t="n"/>
-      <c r="F7" s="6" t="n">
-        <v>46240</v>
-      </c>
-      <c r="G7" s="7" t="n"/>
-      <c r="H7" s="5" t="n"/>
-      <c r="I7" s="5" t="inlineStr">
-        <is>
-          <t>Invalid: empty summary</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>reversed-date</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>Reversed date range</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="D8" s="6" t="n">
-        <v>46244</v>
-      </c>
-      <c r="E8" s="7" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="F8" s="6" t="n">
-        <v>46243</v>
-      </c>
-      <c r="G8" s="7" t="n">
-        <v>0.7083333333333334</v>
-      </c>
-      <c r="H8" s="5" t="inlineStr">
-        <is>
-          <t>Office</t>
-        </is>
-      </c>
-      <c r="I8" s="5" t="inlineStr">
-        <is>
-          <t>Invalid: end date before start date</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>reversed-time</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>Reversed time range</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="D9" s="6" t="n">
-        <v>46245</v>
-      </c>
-      <c r="E9" s="7" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="F9" s="6" t="n">
-        <v>46245</v>
-      </c>
-      <c r="G9" s="7" t="n">
-        <v>0.3333333333333333</v>
-      </c>
-      <c r="H9" s="5" t="inlineStr">
-        <is>
-          <t>Office</t>
-        </is>
-      </c>
-      <c r="I9" s="5" t="inlineStr">
-        <is>
-          <t>Invalid: end time before start time</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>shift-rome</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>Duplicate identifier</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="D10" s="6" t="n">
-        <v>46246</v>
-      </c>
-      <c r="E10" s="7" t="n">
-        <v>0.4166666666666667</v>
-      </c>
-      <c r="F10" s="6" t="n">
-        <v>46246</v>
-      </c>
-      <c r="G10" s="7" t="n">
-        <v>0.4583333333333333</v>
-      </c>
-      <c r="H10" s="5" t="inlineStr">
-        <is>
-          <t>Office</t>
-        </is>
-      </c>
-      <c r="I10" s="5" t="inlineStr">
-        <is>
-          <t>Invalid: duplicate ID</t>
-        </is>
-      </c>
+      <c r="I3" s="2" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:I10"/>

</xml_diff>